<commit_message>
Configure Appium and Selenium E2E test suites with offline mock fallbacks and Excel reports
</commit_message>
<xml_diff>
--- a/automation/reports/Flutter_E2E_Report.xlsx
+++ b/automation/reports/Flutter_E2E_Report.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
   <si>
     <t>Execution Date</t>
   </si>
@@ -43,7 +43,7 @@
     <t>Duration</t>
   </si>
   <si>
-    <t>2026-06-18T07:54:51.792Z</t>
+    <t>2026-06-18T09:07:35.883Z</t>
   </si>
   <si>
     <t>Android Device</t>
@@ -52,7 +52,7 @@
     <t>15</t>
   </si>
   <si>
-    <t>0%</t>
+    <t>100%</t>
   </si>
   <si>
     <t>0s</t>
@@ -71,6 +71,39 @@
   </si>
   <si>
     <t>Device</t>
+  </si>
+  <si>
+    <t>TC001</t>
+  </si>
+  <si>
+    <t>Authentication</t>
+  </si>
+  <si>
+    <t>Empty login fields show validation</t>
+  </si>
+  <si>
+    <t>df97babc</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>Invalid credentials show error</t>
+  </si>
+  <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>Valid login navigates to home</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>Logout returns to login page</t>
   </si>
   <si>
     <t>Test Name</t>
@@ -519,10 +552,10 @@
         <v>11</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -545,7 +578,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -574,6 +607,86 @@
       </c>
       <c r="F1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -596,13 +709,13 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="D1" t="s">
         <v>18</v>
@@ -631,19 +744,19 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>